<commit_message>
Improve Runner content sync and UI state handling
</commit_message>
<xml_diff>
--- a/runner/賽事/人工補充.xlsx
+++ b/runner/賽事/人工補充.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE27958-E854-4B62-95B8-ECA2B2FAC383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="人工補充" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="人工補充" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1012" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="389">
   <si>
     <t>賽事名稱</t>
   </si>
@@ -1164,33 +1160,40 @@
   </si>
   <si>
     <t>人工查證：來源頁全馬與半馬同時起跑（06:30，原資料漏抓這兩組，只有 10K/5K）。</t>
+  </si>
+  <si>
+    <t>2027 第九屆臺中資訊盃公益馬拉松</t>
+  </si>
+  <si>
+    <t>2027-01-24</t>
+  </si>
+  <si>
+    <t>42.195km / 21.0975km / 12km / 5km</t>
+  </si>
+  <si>
+    <t>{"全馬":"06:30","半馬":"06:40","12K":"06:45","5K":"06:55"}</t>
+  </si>
+  <si>
+    <t>2026-07-16</t>
+  </si>
+  <si>
+    <t>人工查證：使用者提供官方活動時程截圖，確認只有全馬、半馬、12K、5K四組及各組起跑時間；移除錯誤的10K與3K，並統一開跑組別顯示名稱。</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="新細明體"/>
-      <family val="3"/>
-      <charset val="136"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1220,7 +1223,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1556,33 +1559,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:V47"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="80.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="137.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="100.375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="255.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="70.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="76.25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="130.375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="107.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="70.625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="188.625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="59.375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="35.125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="188.375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="220.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
+    <col min="7" max="8" width="30" customWidth="1"/>
+    <col min="9" max="12" width="24" customWidth="1"/>
+    <col min="13" max="15" width="20" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="40" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="21" max="21" width="12" customWidth="1"/>
+    <col min="22" max="22" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1650,7 +1647,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1718,7 +1715,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1786,7 +1783,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -1854,7 +1851,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -1922,7 +1919,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -1990,7 +1987,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>77</v>
       </c>
@@ -2058,7 +2055,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -2126,7 +2123,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>106</v>
       </c>
@@ -2194,7 +2191,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>120</v>
       </c>
@@ -2262,7 +2259,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>121</v>
       </c>
@@ -2330,7 +2327,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>133</v>
       </c>
@@ -2398,7 +2395,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>144</v>
       </c>
@@ -2466,7 +2463,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>153</v>
       </c>
@@ -2534,7 +2531,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>163</v>
       </c>
@@ -2602,7 +2599,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>176</v>
       </c>
@@ -2670,7 +2667,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>188</v>
       </c>
@@ -2738,7 +2735,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>199</v>
       </c>
@@ -2806,7 +2803,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>211</v>
       </c>
@@ -2874,7 +2871,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>220</v>
       </c>
@@ -2942,7 +2939,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>232</v>
       </c>
@@ -3010,7 +3007,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>242</v>
       </c>
@@ -3078,7 +3075,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>252</v>
       </c>
@@ -3146,7 +3143,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>264</v>
       </c>
@@ -3214,7 +3211,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>274</v>
       </c>
@@ -3282,7 +3279,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>281</v>
       </c>
@@ -3350,7 +3347,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>286</v>
       </c>
@@ -3418,7 +3415,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>299</v>
       </c>
@@ -3486,7 +3483,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>306</v>
       </c>
@@ -3554,7 +3551,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>310</v>
       </c>
@@ -3622,7 +3619,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>313</v>
       </c>
@@ -3690,7 +3687,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>318</v>
       </c>
@@ -3758,7 +3755,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>323</v>
       </c>
@@ -3826,7 +3823,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>328</v>
       </c>
@@ -3894,7 +3891,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>333</v>
       </c>
@@ -3962,7 +3959,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>339</v>
       </c>
@@ -4030,7 +4027,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>344</v>
       </c>
@@ -4098,7 +4095,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>348</v>
       </c>
@@ -4166,7 +4163,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>354</v>
       </c>
@@ -4234,7 +4231,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>358</v>
       </c>
@@ -4302,7 +4299,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>363</v>
       </c>
@@ -4370,7 +4367,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>366</v>
       </c>
@@ -4438,7 +4435,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>369</v>
       </c>
@@ -4506,7 +4503,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>372</v>
       </c>
@@ -4574,7 +4571,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>376</v>
       </c>
@@ -4642,7 +4639,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>380</v>
       </c>
@@ -4710,10 +4707,77 @@
         <v>382</v>
       </c>
     </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>383</v>
+      </c>
+      <c r="B47" t="s">
+        <v>384</v>
+      </c>
+      <c r="C47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" t="s">
+        <v>26</v>
+      </c>
+      <c r="E47" t="s">
+        <v>26</v>
+      </c>
+      <c r="F47" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" t="s">
+        <v>26</v>
+      </c>
+      <c r="H47" t="s">
+        <v>26</v>
+      </c>
+      <c r="I47" t="s">
+        <v>26</v>
+      </c>
+      <c r="J47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K47" t="s">
+        <v>26</v>
+      </c>
+      <c r="L47" t="s">
+        <v>26</v>
+      </c>
+      <c r="M47" t="s">
+        <v>26</v>
+      </c>
+      <c r="N47" t="s">
+        <v>26</v>
+      </c>
+      <c r="O47" t="s">
+        <v>26</v>
+      </c>
+      <c r="P47" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>26</v>
+      </c>
+      <c r="R47" t="s">
+        <v>385</v>
+      </c>
+      <c r="S47" t="s">
+        <v>386</v>
+      </c>
+      <c r="T47" t="s">
+        <v>26</v>
+      </c>
+      <c r="U47" t="s">
+        <v>387</v>
+      </c>
+      <c r="V47" t="s">
+        <v>388</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <autoFilter ref="A1:V1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>